<commit_message>
Updated compact data with target and source
</commit_message>
<xml_diff>
--- a/dataset/yoruba_sarcasm_data_compact.xlsx
+++ b/dataset/yoruba_sarcasm_data_compact.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
   <workbookPr hidePivotFieldList="1"/>
-  <xr:revisionPtr revIDLastSave="828" documentId="8_{CB3F791A-67BD-4899-88B8-2B5492581178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B877C3D-6841-49CF-92EA-9C289E83939E}"/>
+  <xr:revisionPtr revIDLastSave="829" documentId="8_{CB3F791A-67BD-4899-88B8-2B5492581178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A8997C3-5458-4AB6-B6FC-A835007024A6}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -90,7 +90,7 @@
     <t>A tọrọ owó lọwọ yín, ẹ sì ní kí a wáa gba nílé, èwo ló wáá fa ẹ̀wọ̀n?</t>
   </si>
   <si>
-    <t>Ọmọ náà pupa bíi tááyà ọkọ</t>
+    <t>Ọmọ náà pupa bíi tááyà ọkọ̀</t>
   </si>
   <si>
     <t>Crowdsourcing</t>

</xml_diff>